<commit_message>
Added ATAC-seq computational analysis template
</commit_message>
<xml_diff>
--- a/templates/community/GreenRobust/ATAC-seq_computational_analysis_v0.0.1.xlsx
+++ b/templates/community/GreenRobust/ATAC-seq_computational_analysis_v0.0.1.xlsx
@@ -242,7 +242,7 @@
     <t xml:space="preserve">Term Accession Number () </t>
   </si>
   <si>
-    <t>Output [Sample Name]</t>
+    <t>Output [Data]</t>
   </si>
   <si>
     <t/>
@@ -350,7 +350,7 @@
     <tableColumn id="20" name="Parameter [peak caller]" totalsRowFunction="none"/>
     <tableColumn id="21" name="Term Source REF () " totalsRowFunction="none"/>
     <tableColumn id="22" name="Term Accession Number () " totalsRowFunction="none"/>
-    <tableColumn id="23" name="Output [Sample Name]" totalsRowFunction="none"/>
+    <tableColumn id="23" name="Output [Data]" totalsRowFunction="none"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>